<commit_message>
Diciembre: la Posada pasa al miércoles 16; el lunes 14 vuelve a ser junta normal
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/calendario-el-vive.xlsx
+++ b/datos/calendario-el-vive.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J55"/>
+  <dimension ref="A1:J56"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2341,15 +2341,19 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Especial</t>
+          <t>Lunes de Junta</t>
         </is>
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>Posada durante la junta</t>
-        </is>
-      </c>
-      <c r="F54" s="2" t="n"/>
+          <t>Junta de Comunidad / INI</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>8:00 p.m.</t>
+        </is>
+      </c>
       <c r="G54" s="3" t="inlineStr">
         <is>
           <t>Última junta del mes de diciembre.</t>
@@ -2366,11 +2370,11 @@
         </is>
       </c>
       <c r="B55" s="2" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Jue</t>
+          <t>Mié</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
@@ -2380,7 +2384,7 @@
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>Última Hora Santa del año</t>
+          <t>Posada</t>
         </is>
       </c>
       <c r="F55" s="2" t="n"/>
@@ -2389,13 +2393,43 @@
       <c r="I55" s="3" t="n"/>
       <c r="J55" s="2" t="n"/>
     </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Jue</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>Especial</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>Última Hora Santa del año</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="n"/>
+      <c r="G56" s="3" t="n"/>
+      <c r="H56" s="2" t="n"/>
+      <c r="I56" s="3" t="n"/>
+      <c r="J56" s="2" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H56"/>
   <dataValidations count="4">
-    <dataValidation sqref="D2:D12 D14 D16:D23 D25:D56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="D2:D56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Lunes de Junta,Apostolado,Misa,Matrimonios · KIDS · Juntas,Económica,Especial"</formula1>
     </dataValidation>
-    <dataValidation sqref="D13 D15 D24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="D2:D56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Junta de Consejo,Apostolado,Misa,Matrimonios · KIDS · Juntas,Económica,Especial"</formula1>
     </dataValidation>
     <dataValidation sqref="A2:A56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">

</xml_diff>

<commit_message>
@ Noviembre: se cancela la Entrega de boletos de la Mega Rifa del lunes 2
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
@
</commit_message>
<xml_diff>
--- a/datos/calendario-el-vive.xlsx
+++ b/datos/calendario-el-vive.xlsx
@@ -2,17 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calendario" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Calendario'!$A$1:$H$56</definedName>
-  </definedNames>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -28,23 +27,17 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <family val="2"/>
       <b val="1"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <family val="2"/>
       <b val="1"/>
-      <color rgb="FF6E1E3C"/>
+      <color rgb="006E1E3C"/>
       <sz val="14"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <color rgb="FF333333"/>
+      <color rgb="00333333"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -57,7 +50,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF6E1E3C"/>
+        <fgColor rgb="006E1E3C"/>
       </patternFill>
     </fill>
   </fills>
@@ -71,18 +64,17 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFE2DAD6"/>
+        <color rgb="00E2DAD6"/>
       </left>
       <right style="thin">
-        <color rgb="FFE2DAD6"/>
+        <color rgb="00E2DAD6"/>
       </right>
       <top style="thin">
-        <color rgb="FFE2DAD6"/>
+        <color rgb="00E2DAD6"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFE2DAD6"/>
+        <color rgb="00E2DAD6"/>
       </bottom>
-      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -107,7 +99,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -470,8 +462,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J55"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <dimension ref="A1:J54"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
@@ -479,13 +471,13 @@
     <col width="26" customWidth="1" min="4" max="4"/>
     <col width="48" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="55.140625" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="38" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="21.95" customHeight="1">
+    <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Mes</t>
@@ -566,12 +558,12 @@
           <t>8:00 p.m.</t>
         </is>
       </c>
-      <c r="G2" s="3" t="n"/>
-      <c r="H2" s="2" t="n"/>
-      <c r="I2" s="3" t="n"/>
-      <c r="J2" s="2" t="n"/>
-    </row>
-    <row r="3" ht="30" customHeight="1">
+      <c r="G2" s="3" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="3" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Junio</t>
@@ -600,10 +592,10 @@
           <t>8:00 p.m.</t>
         </is>
       </c>
-      <c r="G3" s="3" t="n"/>
-      <c r="H3" s="2" t="n"/>
-      <c r="I3" s="3" t="n"/>
-      <c r="J3" s="2" t="n"/>
+      <c r="G3" s="3" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="3" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -634,10 +626,10 @@
           <t>8:00 p.m.</t>
         </is>
       </c>
-      <c r="G4" s="3" t="n"/>
-      <c r="H4" s="2" t="n"/>
-      <c r="I4" s="3" t="n"/>
-      <c r="J4" s="2" t="n"/>
+      <c r="G4" s="3" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="3" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -668,10 +660,10 @@
           <t>8:00 p.m.</t>
         </is>
       </c>
-      <c r="G5" s="3" t="n"/>
-      <c r="H5" s="2" t="n"/>
-      <c r="I5" s="3" t="n"/>
-      <c r="J5" s="2" t="n"/>
+      <c r="G5" s="3" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="3" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -702,12 +694,12 @@
           <t>8:00 p.m.</t>
         </is>
       </c>
-      <c r="G6" s="3" t="n"/>
-      <c r="H6" s="2" t="n"/>
-      <c r="I6" s="3" t="n"/>
-      <c r="J6" s="2" t="n"/>
-    </row>
-    <row r="7" ht="30" customHeight="1">
+      <c r="G6" s="3" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="3" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Julio</t>
@@ -718,7 +710,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Mie</t>
+          <t>Mié</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -741,7 +733,7 @@
           <t>Hospital General del Estado (Blvd. Colosio y Quintero Arce)</t>
         </is>
       </c>
-      <c r="H7" s="2" t="n"/>
+      <c r="H7" s="2" t="inlineStr"/>
       <c r="I7" s="3" t="inlineStr">
         <is>
           <t>https://maps.app.goo.gl/wZGdSHUt6B2ged2w8</t>
@@ -787,11 +779,11 @@
           <t>Domingo</t>
         </is>
       </c>
-      <c r="H8" s="2" t="n"/>
-      <c r="I8" s="3" t="n"/>
-      <c r="J8" s="2" t="n"/>
-    </row>
-    <row r="9" ht="30" customHeight="1">
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="3" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Julio</t>
@@ -820,10 +812,10 @@
           <t>8:00 p.m.</t>
         </is>
       </c>
-      <c r="G9" s="3" t="n"/>
-      <c r="H9" s="2" t="n"/>
-      <c r="I9" s="3" t="n"/>
-      <c r="J9" s="2" t="n"/>
+      <c r="G9" s="3" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="3" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -854,10 +846,10 @@
           <t>8:00 p.m.</t>
         </is>
       </c>
-      <c r="G10" s="3" t="n"/>
-      <c r="H10" s="2" t="n"/>
-      <c r="I10" s="3" t="n"/>
-      <c r="J10" s="2" t="n"/>
+      <c r="G10" s="3" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="3" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -866,32 +858,32 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Mié</t>
+          <t>Lun</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Apostolado</t>
+          <t>Lunes de Junta</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Apostolado mensual</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="n"/>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>Lugar por definir</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="n"/>
-      <c r="I11" s="3" t="n"/>
-      <c r="J11" s="2" t="n"/>
+          <t>Junta de Comunidad / INI</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>8:00 p.m.</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="3" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -899,33 +891,39 @@
           <t>Julio</t>
         </is>
       </c>
-      <c r="B12" s="2" t="n">
-        <v>20</v>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>24 – 26</t>
+        </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Lun</t>
+          <t>Vie a Dom</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Lunes de Junta</t>
+          <t>Especial</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Junta de Comunidad / INI</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>8:00 p.m.</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="n"/>
-      <c r="H12" s="2" t="n"/>
-      <c r="I12" s="3" t="n"/>
-      <c r="J12" s="2" t="n"/>
+          <t>Retiro #121 de Monterrey</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr"/>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Nos unimos todos en oración</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -933,39 +931,33 @@
           <t>Julio</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>24 – 26</t>
-        </is>
+      <c r="B13" s="2" t="n">
+        <v>27</v>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Vie a Dom</t>
+          <t>Lun</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Especial</t>
+          <t>Lunes de Junta</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Retiro #121 de Monterrey</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="n"/>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>Nos unimos todos en oración</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="I13" s="3" t="n"/>
-      <c r="J13" s="2" t="n"/>
+          <t>Junta de Comunidad / INI</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>8:00 p.m.</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="3" t="inlineStr"/>
+      <c r="J13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -974,32 +966,32 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Lun</t>
+          <t>Mié</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Lunes de Junta</t>
+          <t>Apostolado</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Junta de Comunidad / INI</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>8:00 p.m.</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="n"/>
-      <c r="H14" s="2" t="n"/>
-      <c r="I14" s="3" t="n"/>
-      <c r="J14" s="2" t="n"/>
+          <t>Apostolado mensual</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr"/>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>Lugar por definir</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr"/>
+      <c r="I14" s="3" t="inlineStr"/>
+      <c r="J14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1027,7 +1019,7 @@
           <t>Retiro #122 de Monterrey</t>
         </is>
       </c>
-      <c r="F15" s="2" t="n"/>
+      <c r="F15" s="2" t="inlineStr"/>
       <c r="G15" s="3" t="inlineStr">
         <is>
           <t>Nos unimos todos en oración</t>
@@ -1038,8 +1030,8 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="I15" s="3" t="n"/>
-      <c r="J15" s="2" t="n"/>
+      <c r="I15" s="3" t="inlineStr"/>
+      <c r="J15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1067,7 +1059,7 @@
           <t>Vacaciones</t>
         </is>
       </c>
-      <c r="F16" s="2" t="n"/>
+      <c r="F16" s="2" t="inlineStr"/>
       <c r="G16" s="3" t="inlineStr">
         <is>
           <t>Del lunes 3 al domingo 16 de agosto.</t>
@@ -1078,10 +1070,10 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="I16" s="3" t="n"/>
-      <c r="J16" s="2" t="n"/>
-    </row>
-    <row r="17" ht="30" customHeight="1">
+      <c r="I16" s="3" t="inlineStr"/>
+      <c r="J16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Agosto</t>
@@ -1105,11 +1097,11 @@
           <t>Misa por el 30.º Aniversario de la Comunidad ÉL VIVE</t>
         </is>
       </c>
-      <c r="F17" s="2" t="n"/>
-      <c r="G17" s="3" t="n"/>
-      <c r="H17" s="2" t="n"/>
-      <c r="I17" s="3" t="n"/>
-      <c r="J17" s="2" t="n"/>
+      <c r="F17" s="2" t="inlineStr"/>
+      <c r="G17" s="3" t="inlineStr"/>
+      <c r="H17" s="2" t="inlineStr"/>
+      <c r="I17" s="3" t="inlineStr"/>
+      <c r="J17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1140,10 +1132,10 @@
           <t>8:00 p.m.</t>
         </is>
       </c>
-      <c r="G18" s="3" t="n"/>
-      <c r="H18" s="2" t="n"/>
-      <c r="I18" s="3" t="n"/>
-      <c r="J18" s="2" t="n"/>
+      <c r="G18" s="3" t="inlineStr"/>
+      <c r="H18" s="2" t="inlineStr"/>
+      <c r="I18" s="3" t="inlineStr"/>
+      <c r="J18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1169,15 +1161,15 @@
           <t>Apostolado mensual</t>
         </is>
       </c>
-      <c r="F19" s="2" t="n"/>
+      <c r="F19" s="2" t="inlineStr"/>
       <c r="G19" s="3" t="inlineStr">
         <is>
           <t>Lugar por definir</t>
         </is>
       </c>
-      <c r="H19" s="2" t="n"/>
-      <c r="I19" s="3" t="n"/>
-      <c r="J19" s="2" t="n"/>
+      <c r="H19" s="2" t="inlineStr"/>
+      <c r="I19" s="3" t="inlineStr"/>
+      <c r="J19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1186,7 +1178,7 @@
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
@@ -1195,12 +1187,12 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Lunes de Junta</t>
+          <t>Matrimonios · KIDS · Juntas</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>Junta de Comunidad / INI</t>
+          <t>Matrimonios ÉL VIVE, KIDS y Juntas de Comunidad e Iniciación</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -1208,10 +1200,10 @@
           <t>8:00 p.m.</t>
         </is>
       </c>
-      <c r="G20" s="3" t="n"/>
-      <c r="H20" s="2" t="n"/>
-      <c r="I20" s="3" t="n"/>
-      <c r="J20" s="2" t="n"/>
+      <c r="G20" s="3" t="inlineStr"/>
+      <c r="H20" s="2" t="inlineStr"/>
+      <c r="I20" s="3" t="inlineStr"/>
+      <c r="J20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1237,11 +1229,11 @@
           <t>Actividad económica chica</t>
         </is>
       </c>
-      <c r="F21" s="2" t="n"/>
-      <c r="G21" s="3" t="n"/>
-      <c r="H21" s="2" t="n"/>
-      <c r="I21" s="3" t="n"/>
-      <c r="J21" s="2" t="n"/>
+      <c r="F21" s="2" t="inlineStr"/>
+      <c r="G21" s="3" t="inlineStr"/>
+      <c r="H21" s="2" t="inlineStr"/>
+      <c r="I21" s="3" t="inlineStr"/>
+      <c r="J21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1277,18 +1269,18 @@
           <t>Domingo</t>
         </is>
       </c>
-      <c r="H22" s="2" t="n"/>
-      <c r="I22" s="3" t="n"/>
-      <c r="J22" s="2" t="n"/>
-    </row>
-    <row r="23" ht="30" customHeight="1">
+      <c r="H22" s="2" t="inlineStr"/>
+      <c r="I22" s="3" t="inlineStr"/>
+      <c r="J22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
           <t>Agosto</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
@@ -1297,12 +1289,12 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Matrimonios · KIDS · Juntas</t>
+          <t>Lunes de Junta</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>Matrimonios ÉL VIVE, KIDS y Juntas de Comunidad e Iniciación</t>
+          <t>Junta de Comunidad / INI</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -1310,10 +1302,10 @@
           <t>8:00 p.m.</t>
         </is>
       </c>
-      <c r="G23" s="3" t="n"/>
-      <c r="H23" s="2" t="n"/>
-      <c r="I23" s="3" t="n"/>
-      <c r="J23" s="2" t="n"/>
+      <c r="G23" s="3" t="inlineStr"/>
+      <c r="H23" s="2" t="inlineStr"/>
+      <c r="I23" s="3" t="inlineStr"/>
+      <c r="J23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1341,7 +1333,7 @@
           <t>Retiro #3 de Chihuahua</t>
         </is>
       </c>
-      <c r="F24" s="2" t="n"/>
+      <c r="F24" s="2" t="inlineStr"/>
       <c r="G24" s="3" t="inlineStr">
         <is>
           <t>Nos unimos todos en oración</t>
@@ -1352,8 +1344,8 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="I24" s="3" t="n"/>
-      <c r="J24" s="2" t="n"/>
+      <c r="I24" s="3" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1384,10 +1376,10 @@
           <t>8:00 p.m.</t>
         </is>
       </c>
-      <c r="G25" s="3" t="n"/>
-      <c r="H25" s="2" t="n"/>
-      <c r="I25" s="3" t="n"/>
-      <c r="J25" s="2" t="n"/>
+      <c r="G25" s="3" t="inlineStr"/>
+      <c r="H25" s="2" t="inlineStr"/>
+      <c r="I25" s="3" t="inlineStr"/>
+      <c r="J25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1418,10 +1410,10 @@
           <t>8:00 p.m.</t>
         </is>
       </c>
-      <c r="G26" s="3" t="n"/>
-      <c r="H26" s="2" t="n"/>
-      <c r="I26" s="3" t="n"/>
-      <c r="J26" s="2" t="n"/>
+      <c r="G26" s="3" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr"/>
+      <c r="I26" s="3" t="inlineStr"/>
+      <c r="J26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1447,11 +1439,11 @@
           <t>Kermés de la Parroquia La Resurrección</t>
         </is>
       </c>
-      <c r="F27" s="2" t="n"/>
-      <c r="G27" s="3" t="n"/>
-      <c r="H27" s="2" t="n"/>
-      <c r="I27" s="3" t="n"/>
-      <c r="J27" s="2" t="n"/>
+      <c r="F27" s="2" t="inlineStr"/>
+      <c r="G27" s="3" t="inlineStr"/>
+      <c r="H27" s="2" t="inlineStr"/>
+      <c r="I27" s="3" t="inlineStr"/>
+      <c r="J27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1460,32 +1452,32 @@
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Mié</t>
+          <t>Lun</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Apostolado</t>
+          <t>Lunes de Junta</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>Apostolado mensual</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="n"/>
-      <c r="G28" s="3" t="inlineStr">
-        <is>
-          <t>Lugar por definir</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="n"/>
-      <c r="I28" s="3" t="n"/>
-      <c r="J28" s="2" t="n"/>
+          <t>Junta de Comunidad / INI</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>8:00 p.m.</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr"/>
+      <c r="H28" s="2" t="inlineStr"/>
+      <c r="I28" s="3" t="inlineStr"/>
+      <c r="J28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1494,32 +1486,32 @@
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Lun</t>
+          <t>Mié</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Lunes de Junta</t>
+          <t>Apostolado</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>Junta de Comunidad / INI</t>
-        </is>
-      </c>
-      <c r="F29" s="2" t="inlineStr">
-        <is>
-          <t>8:00 p.m.</t>
-        </is>
-      </c>
-      <c r="G29" s="3" t="n"/>
-      <c r="H29" s="2" t="n"/>
-      <c r="I29" s="3" t="n"/>
-      <c r="J29" s="2" t="n"/>
+          <t>Apostolado mensual</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr"/>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>Lugar por definir</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr"/>
+      <c r="I29" s="3" t="inlineStr"/>
+      <c r="J29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1555,9 +1547,9 @@
           <t>Domingo</t>
         </is>
       </c>
-      <c r="H30" s="2" t="n"/>
-      <c r="I30" s="3" t="n"/>
-      <c r="J30" s="2" t="n"/>
+      <c r="H30" s="2" t="inlineStr"/>
+      <c r="I30" s="3" t="inlineStr"/>
+      <c r="J30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1588,12 +1580,12 @@
           <t>8:00 p.m.</t>
         </is>
       </c>
-      <c r="G31" s="3" t="n"/>
-      <c r="H31" s="2" t="n"/>
-      <c r="I31" s="3" t="n"/>
-      <c r="J31" s="2" t="n"/>
-    </row>
-    <row r="32" ht="30" customHeight="1">
+      <c r="G31" s="3" t="inlineStr"/>
+      <c r="H31" s="2" t="inlineStr"/>
+      <c r="I31" s="3" t="inlineStr"/>
+      <c r="J31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
           <t>Octubre</t>
@@ -1622,10 +1614,10 @@
           <t>8:00 p.m.</t>
         </is>
       </c>
-      <c r="G32" s="3" t="n"/>
-      <c r="H32" s="2" t="n"/>
-      <c r="I32" s="3" t="n"/>
-      <c r="J32" s="2" t="n"/>
+      <c r="G32" s="3" t="inlineStr"/>
+      <c r="H32" s="2" t="inlineStr"/>
+      <c r="I32" s="3" t="inlineStr"/>
+      <c r="J32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1651,17 +1643,17 @@
           <t>Primera limpieza de rancho con Comunidad de Iniciación 1</t>
         </is>
       </c>
-      <c r="F33" s="2" t="n"/>
+      <c r="F33" s="2" t="inlineStr"/>
       <c r="G33" s="3" t="inlineStr">
         <is>
           <t>Incluye un momento de convivencia, oración y encuentro en el rancho.</t>
         </is>
       </c>
-      <c r="H33" s="2" t="n"/>
-      <c r="I33" s="3" t="n"/>
-      <c r="J33" s="2" t="n"/>
-    </row>
-    <row r="34" ht="30" customHeight="1">
+      <c r="H33" s="2" t="inlineStr"/>
+      <c r="I33" s="3" t="inlineStr"/>
+      <c r="J33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
           <t>Octubre</t>
@@ -1690,10 +1682,10 @@
           <t>8:00 p.m.</t>
         </is>
       </c>
-      <c r="G34" s="3" t="n"/>
-      <c r="H34" s="2" t="n"/>
-      <c r="I34" s="3" t="n"/>
-      <c r="J34" s="2" t="n"/>
+      <c r="G34" s="3" t="inlineStr"/>
+      <c r="H34" s="2" t="inlineStr"/>
+      <c r="I34" s="3" t="inlineStr"/>
+      <c r="J34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -1719,15 +1711,15 @@
           <t>Apostolado mensual</t>
         </is>
       </c>
-      <c r="F35" s="2" t="n"/>
+      <c r="F35" s="2" t="inlineStr"/>
       <c r="G35" s="3" t="inlineStr">
         <is>
           <t>Lugar por definir</t>
         </is>
       </c>
-      <c r="H35" s="2" t="n"/>
-      <c r="I35" s="3" t="n"/>
-      <c r="J35" s="2" t="n"/>
+      <c r="H35" s="2" t="inlineStr"/>
+      <c r="I35" s="3" t="inlineStr"/>
+      <c r="J35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1758,10 +1750,10 @@
           <t>8:00 p.m.</t>
         </is>
       </c>
-      <c r="G36" s="3" t="n"/>
-      <c r="H36" s="2" t="n"/>
-      <c r="I36" s="3" t="n"/>
-      <c r="J36" s="2" t="n"/>
+      <c r="G36" s="3" t="inlineStr"/>
+      <c r="H36" s="2" t="inlineStr"/>
+      <c r="I36" s="3" t="inlineStr"/>
+      <c r="J36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -1787,11 +1779,11 @@
           <t>Actividad económica grande (Conferencias)</t>
         </is>
       </c>
-      <c r="F37" s="2" t="n"/>
-      <c r="G37" s="3" t="n"/>
-      <c r="H37" s="2" t="n"/>
-      <c r="I37" s="3" t="n"/>
-      <c r="J37" s="2" t="n"/>
+      <c r="F37" s="2" t="inlineStr"/>
+      <c r="G37" s="3" t="inlineStr"/>
+      <c r="H37" s="2" t="inlineStr"/>
+      <c r="I37" s="3" t="inlineStr"/>
+      <c r="J37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -1827,9 +1819,9 @@
           <t>Domingo</t>
         </is>
       </c>
-      <c r="H38" s="2" t="n"/>
-      <c r="I38" s="3" t="n"/>
-      <c r="J38" s="2" t="n"/>
+      <c r="H38" s="2" t="inlineStr"/>
+      <c r="I38" s="3" t="inlineStr"/>
+      <c r="J38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -1860,12 +1852,12 @@
           <t>8:00 p.m.</t>
         </is>
       </c>
-      <c r="G39" s="3" t="n"/>
-      <c r="H39" s="2" t="n"/>
-      <c r="I39" s="3" t="n"/>
-      <c r="J39" s="2" t="n"/>
-    </row>
-    <row r="40" ht="30" customHeight="1">
+      <c r="G39" s="3" t="inlineStr"/>
+      <c r="H39" s="2" t="inlineStr"/>
+      <c r="I39" s="3" t="inlineStr"/>
+      <c r="J39" s="2" t="inlineStr"/>
+    </row>
+    <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
           <t>Noviembre</t>
@@ -1894,10 +1886,10 @@
           <t>8:00 p.m.</t>
         </is>
       </c>
-      <c r="G40" s="3" t="n"/>
-      <c r="H40" s="2" t="n"/>
-      <c r="I40" s="3" t="n"/>
-      <c r="J40" s="2" t="n"/>
+      <c r="G40" s="3" t="inlineStr"/>
+      <c r="H40" s="2" t="inlineStr"/>
+      <c r="I40" s="3" t="inlineStr"/>
+      <c r="J40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -1906,7 +1898,7 @@
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
@@ -1915,19 +1907,23 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Económica</t>
+          <t>Lunes de Junta</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>Entrega de boletos de la Mega Rifa</t>
-        </is>
-      </c>
-      <c r="F41" s="2" t="n"/>
-      <c r="G41" s="3" t="n"/>
-      <c r="H41" s="2" t="n"/>
-      <c r="I41" s="3" t="n"/>
-      <c r="J41" s="2" t="n"/>
+          <t>Junta de Comunidad / INI</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>8:00 p.m.</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr"/>
+      <c r="H41" s="2" t="inlineStr"/>
+      <c r="I41" s="3" t="inlineStr"/>
+      <c r="J41" s="2" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -1953,15 +1949,15 @@
           <t>Apostolado mensual</t>
         </is>
       </c>
-      <c r="F42" s="2" t="n"/>
+      <c r="F42" s="2" t="inlineStr"/>
       <c r="G42" s="3" t="inlineStr">
         <is>
           <t>Lugar por definir</t>
         </is>
       </c>
-      <c r="H42" s="2" t="n"/>
-      <c r="I42" s="3" t="n"/>
-      <c r="J42" s="2" t="n"/>
+      <c r="H42" s="2" t="inlineStr"/>
+      <c r="I42" s="3" t="inlineStr"/>
+      <c r="J42" s="2" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -1970,32 +1966,36 @@
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Lun</t>
+          <t>Dom</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Lunes de Junta</t>
+          <t>Misa</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>Junta de Comunidad / INI</t>
+          <t>Misa mensual y convivencia con KIDS</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>8:00 p.m.</t>
-        </is>
-      </c>
-      <c r="G43" s="3" t="n"/>
-      <c r="H43" s="2" t="n"/>
-      <c r="I43" s="3" t="n"/>
-      <c r="J43" s="2" t="n"/>
+          <t>5:00 p.m.</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>(O apostolado con KIDS, por definir.)</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr"/>
+      <c r="I43" s="3" t="inlineStr"/>
+      <c r="J43" s="2" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -2004,36 +2004,32 @@
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Dom</t>
+          <t>Lun</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Misa</t>
+          <t>Lunes de Junta</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>Misa mensual y convivencia con KIDS</t>
+          <t>Junta de Comunidad / INI</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>5:00 p.m.</t>
-        </is>
-      </c>
-      <c r="G44" s="3" t="inlineStr">
-        <is>
-          <t>(O apostolado con KIDS, por definir.)</t>
-        </is>
-      </c>
-      <c r="H44" s="2" t="n"/>
-      <c r="I44" s="3" t="n"/>
-      <c r="J44" s="2" t="n"/>
+          <t>8:00 p.m.</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr"/>
+      <c r="H44" s="2" t="inlineStr"/>
+      <c r="I44" s="3" t="inlineStr"/>
+      <c r="J44" s="2" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -2042,7 +2038,7 @@
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
@@ -2051,12 +2047,12 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Lunes de Junta</t>
+          <t>Matrimonios · KIDS · Juntas</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>Junta de Comunidad / INI</t>
+          <t>Matrimonios ÉL VIVE, KIDS y Juntas de Comunidad e Iniciación</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -2064,10 +2060,10 @@
           <t>8:00 p.m.</t>
         </is>
       </c>
-      <c r="G45" s="3" t="n"/>
-      <c r="H45" s="2" t="n"/>
-      <c r="I45" s="3" t="n"/>
-      <c r="J45" s="2" t="n"/>
+      <c r="G45" s="3" t="inlineStr"/>
+      <c r="H45" s="2" t="inlineStr"/>
+      <c r="I45" s="3" t="inlineStr"/>
+      <c r="J45" s="2" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -2076,71 +2072,71 @@
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Lun</t>
+          <t>Sáb</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Matrimonios · KIDS · Juntas</t>
+          <t>Especial</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>Matrimonios ÉL VIVE, KIDS y Juntas de Comunidad e Iniciación</t>
-        </is>
-      </c>
-      <c r="F46" s="2" t="inlineStr">
-        <is>
-          <t>8:00 p.m.</t>
-        </is>
-      </c>
-      <c r="G46" s="3" t="n"/>
-      <c r="H46" s="2" t="n"/>
-      <c r="I46" s="3" t="n"/>
-      <c r="J46" s="2" t="n"/>
-    </row>
-    <row r="47" ht="30" customHeight="1">
+          <t>Limpieza de rancho</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr"/>
+      <c r="G46" s="3" t="inlineStr"/>
+      <c r="H46" s="2" t="inlineStr"/>
+      <c r="I46" s="3" t="inlineStr"/>
+      <c r="J46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
           <t>Noviembre</t>
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Sáb</t>
+          <t>Lun</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Especial</t>
+          <t>Lunes de Junta</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>Limpieza de rancho</t>
-        </is>
-      </c>
-      <c r="F47" s="2" t="n"/>
-      <c r="G47" s="3" t="n"/>
-      <c r="H47" s="2" t="n"/>
-      <c r="I47" s="3" t="n"/>
-      <c r="J47" s="2" t="n"/>
+          <t>Junta de Comunidad / INI</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>8:00 p.m.</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr"/>
+      <c r="H47" s="2" t="inlineStr"/>
+      <c r="I47" s="3" t="inlineStr"/>
+      <c r="J47" s="2" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Noviembre</t>
+          <t>Diciembre</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>30</v>
+        <v>7</v>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
@@ -2162,10 +2158,10 @@
           <t>8:00 p.m.</t>
         </is>
       </c>
-      <c r="G48" s="3" t="n"/>
-      <c r="H48" s="2" t="n"/>
-      <c r="I48" s="3" t="n"/>
-      <c r="J48" s="2" t="n"/>
+      <c r="G48" s="3" t="inlineStr"/>
+      <c r="H48" s="2" t="inlineStr"/>
+      <c r="I48" s="3" t="inlineStr"/>
+      <c r="J48" s="2" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -2191,15 +2187,15 @@
           <t>Apostolado mensual</t>
         </is>
       </c>
-      <c r="F49" s="2" t="n"/>
+      <c r="F49" s="2" t="inlineStr"/>
       <c r="G49" s="3" t="inlineStr">
         <is>
           <t>Lugar por definir</t>
         </is>
       </c>
-      <c r="H49" s="2" t="n"/>
-      <c r="I49" s="3" t="n"/>
-      <c r="J49" s="2" t="n"/>
+      <c r="H49" s="2" t="inlineStr"/>
+      <c r="I49" s="3" t="inlineStr"/>
+      <c r="J49" s="2" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -2208,32 +2204,28 @@
         </is>
       </c>
       <c r="B50" s="2" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Lun</t>
+          <t>Vie</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Lunes de Junta</t>
+          <t>Especial</t>
         </is>
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>Junta de Comunidad / INI</t>
-        </is>
-      </c>
-      <c r="F50" s="2" t="inlineStr">
-        <is>
-          <t>8:00 p.m.</t>
-        </is>
-      </c>
-      <c r="G50" s="3" t="n"/>
-      <c r="H50" s="2" t="n"/>
-      <c r="I50" s="3" t="n"/>
-      <c r="J50" s="2" t="n"/>
+          <t>Peregrinación</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr"/>
+      <c r="G50" s="3" t="inlineStr"/>
+      <c r="H50" s="2" t="inlineStr"/>
+      <c r="I50" s="3" t="inlineStr"/>
+      <c r="J50" s="2" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -2242,11 +2234,11 @@
         </is>
       </c>
       <c r="B51" s="2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Vie</t>
+          <t>Sáb</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -2256,14 +2248,14 @@
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>Peregrinación</t>
-        </is>
-      </c>
-      <c r="F51" s="2" t="n"/>
-      <c r="G51" s="3" t="n"/>
-      <c r="H51" s="2" t="n"/>
-      <c r="I51" s="3" t="n"/>
-      <c r="J51" s="2" t="n"/>
+          <t>Día de la Virgen, misa y Posada KIDS</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr"/>
+      <c r="G51" s="3" t="inlineStr"/>
+      <c r="H51" s="2" t="inlineStr"/>
+      <c r="I51" s="3" t="inlineStr"/>
+      <c r="J51" s="2" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -2272,28 +2264,36 @@
         </is>
       </c>
       <c r="B52" s="2" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Sáb</t>
+          <t>Lun</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Especial</t>
+          <t>Lunes de Junta</t>
         </is>
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t>Día de la Virgen, misa y Posada KIDS</t>
-        </is>
-      </c>
-      <c r="F52" s="2" t="n"/>
-      <c r="G52" s="3" t="n"/>
-      <c r="H52" s="2" t="n"/>
-      <c r="I52" s="3" t="n"/>
-      <c r="J52" s="2" t="n"/>
+          <t>Junta de Comunidad / INI</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>8:00 p.m.</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>Última junta del mes de diciembre.</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr"/>
+      <c r="I52" s="3" t="inlineStr"/>
+      <c r="J52" s="2" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -2302,36 +2302,28 @@
         </is>
       </c>
       <c r="B53" s="2" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Lun</t>
+          <t>Mié</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Lunes de Junta</t>
+          <t>Especial</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>Junta de Comunidad / INI</t>
-        </is>
-      </c>
-      <c r="F53" s="2" t="inlineStr">
-        <is>
-          <t>8:00 p.m.</t>
-        </is>
-      </c>
-      <c r="G53" s="3" t="inlineStr">
-        <is>
-          <t>Última junta del mes de diciembre.</t>
-        </is>
-      </c>
-      <c r="H53" s="2" t="n"/>
-      <c r="I53" s="3" t="n"/>
-      <c r="J53" s="2" t="n"/>
+          <t>Posada</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr"/>
+      <c r="G53" s="3" t="inlineStr"/>
+      <c r="H53" s="2" t="inlineStr"/>
+      <c r="I53" s="3" t="inlineStr"/>
+      <c r="J53" s="2" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -2340,11 +2332,11 @@
         </is>
       </c>
       <c r="B54" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Mié</t>
+          <t>Jue</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
@@ -2354,58 +2346,27 @@
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>Posada</t>
-        </is>
-      </c>
-      <c r="F54" s="2" t="n"/>
-      <c r="G54" s="3" t="n"/>
-      <c r="H54" s="2" t="n"/>
-      <c r="I54" s="3" t="n"/>
-      <c r="J54" s="2" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="2" t="inlineStr">
-        <is>
-          <t>Diciembre</t>
-        </is>
-      </c>
-      <c r="B55" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="C55" s="2" t="inlineStr">
-        <is>
-          <t>Jue</t>
-        </is>
-      </c>
-      <c r="D55" s="2" t="inlineStr">
-        <is>
-          <t>Especial</t>
-        </is>
-      </c>
-      <c r="E55" s="3" t="inlineStr">
-        <is>
           <t>Última Hora Santa del año</t>
         </is>
       </c>
-      <c r="F55" s="2" t="n"/>
-      <c r="G55" s="3" t="n"/>
-      <c r="H55" s="2" t="n"/>
-      <c r="I55" s="3" t="n"/>
-      <c r="J55" s="2" t="n"/>
+      <c r="F54" s="2" t="inlineStr"/>
+      <c r="G54" s="3" t="inlineStr"/>
+      <c r="H54" s="2" t="inlineStr"/>
+      <c r="I54" s="3" t="inlineStr"/>
+      <c r="J54" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H56"/>
   <dataValidations count="4">
-    <dataValidation sqref="D2:D55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="A2:A54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Junio,Julio,Agosto,Septiembre,Octubre,Noviembre,Diciembre"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D2:D54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Lunes de Junta,Apostolado,Misa,Matrimonios · KIDS · Juntas,Económica,Especial"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"Junta de Consejo,Apostolado,Misa,Matrimonios · KIDS · Juntas,Económica,Especial"</formula1>
+    <dataValidation sqref="H2:H54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Sí,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="A2:A55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"Junio,Julio,Agosto,Septiembre,Octubre,Noviembre,Diciembre"</formula1>
-    </dataValidation>
-    <dataValidation sqref="H2:H55 J2:J55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Sí,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2420,12 +2381,12 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:A15"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18.75" customHeight="1">
+    <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
           <t>CALENDARIO ÉL VIVE · Cómo editar</t>
@@ -2433,7 +2394,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="n"/>
+      <c r="A2" s="5" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
@@ -2513,7 +2474,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="n"/>
+      <c r="A14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Diciembre: agrega el Retiro de Compromiso INI #1 (4 – 6), destacado en azul claro
Sigue siendo categoría Especial, pero la tarjeta de la Lista y la barra de la
vista Mes se pintan en azul claro para resaltarlo como el evento del año.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/calendario-el-vive.xlsx
+++ b/datos/calendario-el-vive.xlsx
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J54"/>
+  <dimension ref="A1:J55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2354,6 +2354,42 @@
       <c r="H54" s="2" t="inlineStr"/>
       <c r="I54" s="3" t="inlineStr"/>
       <c r="J54" s="2" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>4 – 6</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Vie a Dom</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Especial</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>Retiro de Compromiso INI #1</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="n"/>
+      <c r="G55" s="3" t="n"/>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I55" s="3" t="n"/>
+      <c r="J55" s="2" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="4">

</xml_diff>

<commit_message>
Octubre: Hora Santa en Ures (2), junta de Matrimonios recorrida al 5, Juntos el 12, Cine ÉL VIVE el 19; Conferencias pasan al 25 nov
- 28 sep: se marca «No hubo junta» (clima): tarjeta en gris, título tachado,
  sin check ni botón de comentarios. Nueva columna «Cancelado (no hubo)» en el Excel.
- 5 oct: pasa a Matrimonios ÉL VIVE, KIDS y Juntas (fecha actualizada).
- Se quitan la limpieza de rancho del 10 oct y la actividad económica del 24 oct.
- 25 nov: Conferencias ÉL VIVE (Económica).

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/calendario-el-vive.xlsx
+++ b/datos/calendario-el-vive.xlsx
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J55"/>
+  <dimension ref="A1:K55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -475,6 +475,7 @@
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="38" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -526,6 +527,11 @@
       <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Reprogramado</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Cancelado (no hubo)</t>
         </is>
       </c>
     </row>
@@ -1580,10 +1586,19 @@
           <t>8:00 p.m.</t>
         </is>
       </c>
-      <c r="G31" s="3" t="inlineStr"/>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>No hubo junta por el clima. Se recorrió al lunes 5 de octubre.</t>
+        </is>
+      </c>
       <c r="H31" s="2" t="inlineStr"/>
       <c r="I31" s="3" t="inlineStr"/>
       <c r="J31" s="2" t="inlineStr"/>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1601,12 +1616,12 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Lunes de Junta</t>
+          <t>Matrimonios · KIDS · Juntas</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>Junta de Comunidad / INI</t>
+          <t>Matrimonios ÉL VIVE, KIDS y Juntas de Comunidad e Iniciación</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -1614,10 +1629,18 @@
           <t>8:00 p.m.</t>
         </is>
       </c>
-      <c r="G32" s="3" t="inlineStr"/>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>Se recorrió del lunes 28 de septiembre (no hubo junta por el clima).</t>
+        </is>
+      </c>
       <c r="H32" s="2" t="inlineStr"/>
       <c r="I32" s="3" t="inlineStr"/>
-      <c r="J32" s="2" t="inlineStr"/>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1626,11 +1649,11 @@
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Sáb</t>
+          <t>Vie</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -1640,18 +1663,14 @@
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>Primera limpieza de rancho con Comunidad de Iniciación 1</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="inlineStr"/>
-      <c r="G33" s="3" t="inlineStr">
-        <is>
-          <t>Incluye un momento de convivencia, oración y encuentro en el rancho.</t>
-        </is>
-      </c>
-      <c r="H33" s="2" t="inlineStr"/>
-      <c r="I33" s="3" t="inlineStr"/>
-      <c r="J33" s="2" t="inlineStr"/>
+          <t>Hora Santa en Ures</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="n"/>
+      <c r="G33" s="3" t="n"/>
+      <c r="H33" s="2" t="n"/>
+      <c r="I33" s="3" t="n"/>
+      <c r="J33" s="2" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1674,7 +1693,7 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>Junta de Comunidad / INI</t>
+          <t>Junta de Comunidad e Iniciación (Juntos)</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -1737,12 +1756,12 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Lunes de Junta</t>
+          <t>Especial</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>Junta de Comunidad / INI</t>
+          <t>Cine ÉL VIVE - The Chosen Cap.1 Temp.6</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -1758,15 +1777,15 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Octubre</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Sáb</t>
+          <t>Mié</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -1776,7 +1795,7 @@
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>Actividad económica grande (Conferencias)</t>
+          <t>Conferencias ÉL VIVE</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Octubre: quita el apostolado del 14 y la nota del 5; la junta cancelada del 28 sep ya no va tachada
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/calendario-el-vive.xlsx
+++ b/datos/calendario-el-vive.xlsx
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K55"/>
+  <dimension ref="A1:K54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1629,11 +1629,7 @@
           <t>8:00 p.m.</t>
         </is>
       </c>
-      <c r="G32" s="3" t="inlineStr">
-        <is>
-          <t>Se recorrió del lunes 28 de septiembre (no hubo junta por el clima).</t>
-        </is>
-      </c>
+      <c r="G32" s="3" t="n"/>
       <c r="H32" s="2" t="inlineStr"/>
       <c r="I32" s="3" t="inlineStr"/>
       <c r="J32" s="2" t="inlineStr">
@@ -1713,29 +1709,29 @@
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Mié</t>
+          <t>Lun</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Apostolado</t>
+          <t>Especial</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>Apostolado mensual</t>
-        </is>
-      </c>
-      <c r="F35" s="2" t="inlineStr"/>
-      <c r="G35" s="3" t="inlineStr">
-        <is>
-          <t>Lugar por definir</t>
-        </is>
-      </c>
+          <t>Cine ÉL VIVE - The Chosen Cap.1 Temp.6</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>8:00 p.m.</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr"/>
       <c r="H35" s="2" t="inlineStr"/>
       <c r="I35" s="3" t="inlineStr"/>
       <c r="J35" s="2" t="inlineStr"/>
@@ -1743,32 +1739,28 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Octubre</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Lun</t>
+          <t>Mié</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Especial</t>
+          <t>Económica</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>Cine ÉL VIVE - The Chosen Cap.1 Temp.6</t>
-        </is>
-      </c>
-      <c r="F36" s="2" t="inlineStr">
-        <is>
-          <t>8:00 p.m.</t>
-        </is>
-      </c>
+          <t>Conferencias ÉL VIVE</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr"/>
       <c r="G36" s="3" t="inlineStr"/>
       <c r="H36" s="2" t="inlineStr"/>
       <c r="I36" s="3" t="inlineStr"/>
@@ -1777,7 +1769,7 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Noviembre</t>
+          <t>Octubre</t>
         </is>
       </c>
       <c r="B37" s="2" t="n">
@@ -1785,21 +1777,29 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Mié</t>
+          <t>Dom</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Económica</t>
+          <t>Misa</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>Conferencias ÉL VIVE</t>
-        </is>
-      </c>
-      <c r="F37" s="2" t="inlineStr"/>
-      <c r="G37" s="3" t="inlineStr"/>
+          <t>Misa mensual</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>5:00 p.m.</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>Domingo</t>
+        </is>
+      </c>
       <c r="H37" s="2" t="inlineStr"/>
       <c r="I37" s="3" t="inlineStr"/>
       <c r="J37" s="2" t="inlineStr"/>
@@ -1811,33 +1811,29 @@
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Dom</t>
+          <t>Lun</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Misa</t>
+          <t>Matrimonios · KIDS · Juntas</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>Misa mensual</t>
+          <t>Matrimonios ÉL VIVE, KIDS y Juntas de Comunidad e Iniciación</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>5:00 p.m.</t>
-        </is>
-      </c>
-      <c r="G38" s="3" t="inlineStr">
-        <is>
-          <t>Domingo</t>
-        </is>
-      </c>
+          <t>8:00 p.m.</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr"/>
       <c r="H38" s="2" t="inlineStr"/>
       <c r="I38" s="3" t="inlineStr"/>
       <c r="J38" s="2" t="inlineStr"/>
@@ -1845,11 +1841,11 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Octubre</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
@@ -1858,12 +1854,12 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Matrimonios · KIDS · Juntas</t>
+          <t>Lunes de Junta</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>Matrimonios ÉL VIVE, KIDS y Juntas de Comunidad e Iniciación</t>
+          <t>Junta de Comunidad / INI</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -1883,7 +1879,7 @@
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
@@ -1917,29 +1913,29 @@
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Lun</t>
+          <t>Sáb</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Lunes de Junta</t>
+          <t>Apostolado</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>Junta de Comunidad / INI</t>
-        </is>
-      </c>
-      <c r="F41" s="2" t="inlineStr">
-        <is>
-          <t>8:00 p.m.</t>
-        </is>
-      </c>
-      <c r="G41" s="3" t="inlineStr"/>
+          <t>Apostolado mensual</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr"/>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>Lugar por definir</t>
+        </is>
+      </c>
       <c r="H41" s="2" t="inlineStr"/>
       <c r="I41" s="3" t="inlineStr"/>
       <c r="J41" s="2" t="inlineStr"/>
@@ -1951,27 +1947,31 @@
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Sáb</t>
+          <t>Dom</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Apostolado</t>
+          <t>Misa</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>Apostolado mensual</t>
-        </is>
-      </c>
-      <c r="F42" s="2" t="inlineStr"/>
+          <t>Misa mensual y convivencia con KIDS</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>5:00 p.m.</t>
+        </is>
+      </c>
       <c r="G42" s="3" t="inlineStr">
         <is>
-          <t>Lugar por definir</t>
+          <t>(O apostolado con KIDS, por definir.)</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr"/>
@@ -1985,33 +1985,29 @@
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Dom</t>
+          <t>Lun</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Misa</t>
+          <t>Lunes de Junta</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>Misa mensual y convivencia con KIDS</t>
+          <t>Junta de Comunidad / INI</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>5:00 p.m.</t>
-        </is>
-      </c>
-      <c r="G43" s="3" t="inlineStr">
-        <is>
-          <t>(O apostolado con KIDS, por definir.)</t>
-        </is>
-      </c>
+          <t>8:00 p.m.</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr"/>
       <c r="H43" s="2" t="inlineStr"/>
       <c r="I43" s="3" t="inlineStr"/>
       <c r="J43" s="2" t="inlineStr"/>
@@ -2023,7 +2019,7 @@
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
@@ -2032,12 +2028,12 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Lunes de Junta</t>
+          <t>Matrimonios · KIDS · Juntas</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>Junta de Comunidad / INI</t>
+          <t>Matrimonios ÉL VIVE, KIDS y Juntas de Comunidad e Iniciación</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -2057,28 +2053,24 @@
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Lun</t>
+          <t>Sáb</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Matrimonios · KIDS · Juntas</t>
+          <t>Especial</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>Matrimonios ÉL VIVE, KIDS y Juntas de Comunidad e Iniciación</t>
-        </is>
-      </c>
-      <c r="F45" s="2" t="inlineStr">
-        <is>
-          <t>8:00 p.m.</t>
-        </is>
-      </c>
+          <t>Limpieza de rancho</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr"/>
       <c r="G45" s="3" t="inlineStr"/>
       <c r="H45" s="2" t="inlineStr"/>
       <c r="I45" s="3" t="inlineStr"/>
@@ -2091,24 +2083,28 @@
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Sáb</t>
+          <t>Lun</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Especial</t>
+          <t>Lunes de Junta</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>Limpieza de rancho</t>
-        </is>
-      </c>
-      <c r="F46" s="2" t="inlineStr"/>
+          <t>Junta de Comunidad / INI</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>8:00 p.m.</t>
+        </is>
+      </c>
       <c r="G46" s="3" t="inlineStr"/>
       <c r="H46" s="2" t="inlineStr"/>
       <c r="I46" s="3" t="inlineStr"/>
@@ -2117,11 +2113,11 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Noviembre</t>
+          <t>Diciembre</t>
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>30</v>
+        <v>7</v>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
@@ -2155,29 +2151,29 @@
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Lun</t>
+          <t>Mié</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Lunes de Junta</t>
+          <t>Apostolado</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>Junta de Comunidad / INI</t>
-        </is>
-      </c>
-      <c r="F48" s="2" t="inlineStr">
-        <is>
-          <t>8:00 p.m.</t>
-        </is>
-      </c>
-      <c r="G48" s="3" t="inlineStr"/>
+          <t>Apostolado mensual</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr"/>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>Lugar por definir</t>
+        </is>
+      </c>
       <c r="H48" s="2" t="inlineStr"/>
       <c r="I48" s="3" t="inlineStr"/>
       <c r="J48" s="2" t="inlineStr"/>
@@ -2189,29 +2185,25 @@
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Mié</t>
+          <t>Vie</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Apostolado</t>
+          <t>Especial</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>Apostolado mensual</t>
+          <t>Peregrinación</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr"/>
-      <c r="G49" s="3" t="inlineStr">
-        <is>
-          <t>Lugar por definir</t>
-        </is>
-      </c>
+      <c r="G49" s="3" t="inlineStr"/>
       <c r="H49" s="2" t="inlineStr"/>
       <c r="I49" s="3" t="inlineStr"/>
       <c r="J49" s="2" t="inlineStr"/>
@@ -2223,11 +2215,11 @@
         </is>
       </c>
       <c r="B50" s="2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Vie</t>
+          <t>Sáb</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
@@ -2237,7 +2229,7 @@
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>Peregrinación</t>
+          <t>Día de la Virgen, misa y Posada KIDS</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr"/>
@@ -2253,25 +2245,33 @@
         </is>
       </c>
       <c r="B51" s="2" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Sáb</t>
+          <t>Lun</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Especial</t>
+          <t>Lunes de Junta</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>Día de la Virgen, misa y Posada KIDS</t>
-        </is>
-      </c>
-      <c r="F51" s="2" t="inlineStr"/>
-      <c r="G51" s="3" t="inlineStr"/>
+          <t>Junta de Comunidad / INI</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>8:00 p.m.</t>
+        </is>
+      </c>
+      <c r="G51" s="3" t="inlineStr">
+        <is>
+          <t>Última junta del mes de diciembre.</t>
+        </is>
+      </c>
       <c r="H51" s="2" t="inlineStr"/>
       <c r="I51" s="3" t="inlineStr"/>
       <c r="J51" s="2" t="inlineStr"/>
@@ -2283,33 +2283,25 @@
         </is>
       </c>
       <c r="B52" s="2" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Lun</t>
+          <t>Mié</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Lunes de Junta</t>
+          <t>Especial</t>
         </is>
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t>Junta de Comunidad / INI</t>
-        </is>
-      </c>
-      <c r="F52" s="2" t="inlineStr">
-        <is>
-          <t>8:00 p.m.</t>
-        </is>
-      </c>
-      <c r="G52" s="3" t="inlineStr">
-        <is>
-          <t>Última junta del mes de diciembre.</t>
-        </is>
-      </c>
+          <t>Posada</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr"/>
+      <c r="G52" s="3" t="inlineStr"/>
       <c r="H52" s="2" t="inlineStr"/>
       <c r="I52" s="3" t="inlineStr"/>
       <c r="J52" s="2" t="inlineStr"/>
@@ -2321,11 +2313,11 @@
         </is>
       </c>
       <c r="B53" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Mié</t>
+          <t>Jue</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
@@ -2335,7 +2327,7 @@
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>Posada</t>
+          <t>Última Hora Santa del año</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr"/>
@@ -2350,12 +2342,14 @@
           <t>Diciembre</t>
         </is>
       </c>
-      <c r="B54" s="2" t="n">
-        <v>17</v>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>4 – 6</t>
+        </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Jue</t>
+          <t>Vie a Dom</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
@@ -2365,50 +2359,18 @@
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>Última Hora Santa del año</t>
-        </is>
-      </c>
-      <c r="F54" s="2" t="inlineStr"/>
-      <c r="G54" s="3" t="inlineStr"/>
-      <c r="H54" s="2" t="inlineStr"/>
-      <c r="I54" s="3" t="inlineStr"/>
-      <c r="J54" s="2" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="2" t="inlineStr">
-        <is>
-          <t>Diciembre</t>
-        </is>
-      </c>
-      <c r="B55" s="2" t="inlineStr">
-        <is>
-          <t>4 – 6</t>
-        </is>
-      </c>
-      <c r="C55" s="2" t="inlineStr">
-        <is>
-          <t>Vie a Dom</t>
-        </is>
-      </c>
-      <c r="D55" s="2" t="inlineStr">
-        <is>
-          <t>Especial</t>
-        </is>
-      </c>
-      <c r="E55" s="3" t="inlineStr">
-        <is>
           <t>Retiro de Compromiso INI #1</t>
         </is>
       </c>
-      <c r="F55" s="2" t="n"/>
-      <c r="G55" s="3" t="n"/>
-      <c r="H55" s="2" t="inlineStr">
+      <c r="F54" s="2" t="n"/>
+      <c r="G54" s="3" t="n"/>
+      <c r="H54" s="2" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="I55" s="3" t="n"/>
-      <c r="J55" s="2" t="n"/>
+      <c r="I54" s="3" t="n"/>
+      <c r="J54" s="2" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="4">

</xml_diff>

<commit_message>
Octubre: agrega Lunada en el Rancho (sáb 24 – dom 25)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/calendario-el-vive.xlsx
+++ b/datos/calendario-el-vive.xlsx
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K54"/>
+  <dimension ref="A1:K55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2371,6 +2371,42 @@
       </c>
       <c r="I54" s="3" t="n"/>
       <c r="J54" s="2" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>Octubre</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>24 – 25</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Sáb a Dom</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Especial</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>Lunada en el Rancho</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="n"/>
+      <c r="G55" s="3" t="n"/>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I55" s="3" t="n"/>
+      <c r="J55" s="2" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="4">

</xml_diff>

<commit_message>
Octubre: agrega Apostolado mensual el sáb 31 (9:00 a.m., Casa Esperanza para niños)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/calendario-el-vive.xlsx
+++ b/datos/calendario-el-vive.xlsx
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K55"/>
+  <dimension ref="A1:K56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2407,6 +2407,41 @@
       </c>
       <c r="I55" s="3" t="n"/>
       <c r="J55" s="2" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Octubre</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>31</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Sáb</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Apostolado</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Apostolado mensual</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>9:00 a.m.</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Casa Esperanza para niños</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="4">

</xml_diff>